<commit_message>
refacto: planinha de riscos atualizada
</commit_message>
<xml_diff>
--- a/Documentações/Planilha de riscos.xlsx
+++ b/Documentações/Planilha de riscos.xlsx
@@ -8,12 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\albuq\Repositorios\ThermoChain\Documentações\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{717AB33A-1055-4879-9C30-AAB66EE8CFEB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05D78B6A-3543-48B9-AC61-E9373C56AC07}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Plan1" sheetId="1" r:id="rId1"/>
+    <sheet name="planinha de risco" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="36">
   <si>
     <t>id</t>
   </si>
@@ -80,6 +80,78 @@
   <si>
     <t>Muito Provável
 (3)</t>
+  </si>
+  <si>
+    <t>Atrasar os entregáveis</t>
+  </si>
+  <si>
+    <t>Algum integrante não comparecer na apresentação</t>
+  </si>
+  <si>
+    <t>Mudar o grupo de posição
+ e não estar todos presentes no momento</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Todos computadores para apresentação estarem mal
+ configurados </t>
+  </si>
+  <si>
+    <t>Algum integrante ficar pouco presente ou ausente nos ensaios para apresentar</t>
+  </si>
+  <si>
+    <t>Parte do grupo estar com dificuldade
+ sobre algum assunto</t>
+  </si>
+  <si>
+    <t>O sensor estar medindo errado por mal configuração</t>
+  </si>
+  <si>
+    <t>1 - Baixa</t>
+  </si>
+  <si>
+    <t>2 - Média</t>
+  </si>
+  <si>
+    <t>1 - baixa</t>
+  </si>
+  <si>
+    <t>3 - Alto</t>
+  </si>
+  <si>
+    <t>1 - Baixo</t>
+  </si>
+  <si>
+    <t>2 - Médio</t>
+  </si>
+  <si>
+    <t>Mitigar</t>
+  </si>
+  <si>
+    <t>Evitar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Integrando todos do grupo no projeto
+ e realizando daily </t>
+  </si>
+  <si>
+    <t>Combinar um hórario de chegada que anteceda, afim de realizar um último ensaio</t>
+  </si>
+  <si>
+    <t>Sair o mais cedo possível eliminando os fatores externos, eliminar compromissos do dia anterior afim de dormir bem e acordar no horário</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Levar pen-drive para backup, verificar computador principal
+ e reserva com 2 horas de antecedência </t>
+  </si>
+  <si>
+    <t>Ter comunicação ativa para que se algum integrante
+ perceber que há dificuldade o grupo apoia-lo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Testar o sensor horas antes </t>
+  </si>
+  <si>
+    <t>Incentivar o compromentimento de todos do grupo</t>
   </si>
 </sst>
 </file>
@@ -142,7 +214,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -165,11 +237,24 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -183,7 +268,6 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -194,6 +278,20 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -474,15 +572,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="D1:P8"/>
+  <dimension ref="D1:P11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="5" max="5" width="21.5703125" customWidth="1"/>
-    <col min="6" max="6" width="31.140625" customWidth="1"/>
+    <col min="5" max="5" width="48.140625" customWidth="1"/>
+    <col min="6" max="6" width="31.28515625" customWidth="1"/>
     <col min="7" max="7" width="22.7109375" customWidth="1"/>
     <col min="8" max="8" width="19" customWidth="1"/>
     <col min="9" max="9" width="16.5703125" customWidth="1"/>
-    <col min="10" max="10" width="34.140625" customWidth="1"/>
+    <col min="10" max="10" width="76.140625" customWidth="1"/>
     <col min="13" max="16" width="13" customWidth="1"/>
   </cols>
   <sheetData>
@@ -510,89 +608,158 @@
       </c>
     </row>
     <row r="2" spans="4:16" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D2" s="1"/>
-      <c r="E2" s="1"/>
-      <c r="F2" s="1"/>
-      <c r="G2" s="1"/>
-      <c r="H2" s="1"/>
-      <c r="I2" s="1"/>
-      <c r="J2" s="1"/>
+      <c r="D2" s="1">
+        <v>1</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="H2" s="6">
+        <v>3</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>29</v>
+      </c>
       <c r="M2" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="3" spans="4:16" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D3" s="1"/>
-      <c r="E3" s="1"/>
-      <c r="F3" s="1"/>
-      <c r="G3" s="1"/>
-      <c r="H3" s="1"/>
-      <c r="I3" s="1"/>
-      <c r="J3" s="1"/>
+      <c r="D3" s="1">
+        <v>2</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="H3" s="7">
+        <v>6</v>
+      </c>
+      <c r="I3" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="J3" s="1" t="s">
+        <v>30</v>
+      </c>
       <c r="M3" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="N3" s="7">
+      <c r="N3" s="6">
         <v>3</v>
       </c>
-      <c r="O3" s="8">
+      <c r="O3" s="7">
         <v>6</v>
       </c>
-      <c r="P3" s="8">
+      <c r="P3" s="7">
         <v>9</v>
       </c>
     </row>
     <row r="4" spans="4:16" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D4" s="1"/>
-      <c r="E4" s="1"/>
-      <c r="F4" s="1"/>
-      <c r="G4" s="1"/>
-      <c r="H4" s="1"/>
-      <c r="I4" s="1"/>
-      <c r="J4" s="1"/>
+      <c r="D4" s="1">
+        <v>3</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="H4" s="5">
+        <v>1</v>
+      </c>
+      <c r="I4" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="J4" s="2" t="s">
+        <v>31</v>
+      </c>
       <c r="M4" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="N4" s="6">
+      <c r="N4" s="5">
         <v>2</v>
       </c>
-      <c r="O4" s="7">
+      <c r="O4" s="6">
         <v>4</v>
       </c>
-      <c r="P4" s="8">
+      <c r="P4" s="7">
         <v>6</v>
       </c>
     </row>
     <row r="5" spans="4:16" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D5" s="1"/>
-      <c r="E5" s="1"/>
-      <c r="F5" s="1"/>
-      <c r="G5" s="1"/>
-      <c r="H5" s="1"/>
-      <c r="I5" s="1"/>
-      <c r="J5" s="1"/>
+      <c r="D5" s="1">
+        <v>4</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="H5" s="6">
+        <v>3</v>
+      </c>
+      <c r="I5" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="J5" s="2" t="s">
+        <v>32</v>
+      </c>
       <c r="M5" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="N5" s="6">
+      <c r="N5" s="5">
         <v>1</v>
       </c>
-      <c r="O5" s="6">
+      <c r="O5" s="5">
         <v>2</v>
       </c>
-      <c r="P5" s="7">
+      <c r="P5" s="6">
         <v>3</v>
       </c>
     </row>
     <row r="6" spans="4:16" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D6" s="1"/>
-      <c r="E6" s="1"/>
-      <c r="F6" s="1"/>
-      <c r="G6" s="1"/>
-      <c r="H6" s="1"/>
-      <c r="I6" s="1"/>
-      <c r="J6" s="1"/>
-      <c r="M6" s="5"/>
+      <c r="D6" s="1">
+        <v>5</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="H6" s="6">
+        <v>4</v>
+      </c>
+      <c r="I6" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="J6" s="1" t="s">
+        <v>35</v>
+      </c>
       <c r="N6" s="2" t="s">
         <v>11</v>
       </c>
@@ -604,23 +771,63 @@
       </c>
     </row>
     <row r="7" spans="4:16" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D7" s="1"/>
-      <c r="E7" s="1"/>
-      <c r="F7" s="1"/>
-      <c r="G7" s="1"/>
-      <c r="H7" s="1"/>
-      <c r="I7" s="1"/>
-      <c r="J7" s="1"/>
+      <c r="D7" s="9">
+        <v>6</v>
+      </c>
+      <c r="E7" s="11" t="s">
+        <v>19</v>
+      </c>
+      <c r="F7" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="G7" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="H7" s="12">
+        <v>3</v>
+      </c>
+      <c r="I7" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="J7" s="11" t="s">
+        <v>33</v>
+      </c>
     </row>
     <row r="8" spans="4:16" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D8" s="1"/>
-      <c r="E8" s="1"/>
-      <c r="F8" s="1"/>
-      <c r="G8" s="1"/>
-      <c r="H8" s="1"/>
-      <c r="I8" s="1"/>
-      <c r="J8" s="1"/>
-      <c r="O8" s="9"/>
+      <c r="D8" s="1">
+        <v>7</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="G8" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="H8" s="7">
+        <v>6</v>
+      </c>
+      <c r="I8" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="J8" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="O8" s="8"/>
+    </row>
+    <row r="9" spans="4:16" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D9" s="13"/>
+      <c r="E9" s="10"/>
+      <c r="F9" s="10"/>
+      <c r="G9" s="10"/>
+      <c r="H9" s="10"/>
+      <c r="I9" s="10"/>
+      <c r="J9" s="10"/>
+    </row>
+    <row r="11" spans="4:16" x14ac:dyDescent="0.25">
+      <c r="J11" s="14"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>